<commit_message>
feat: translate profile templates, cron, and core tools to English
- Translate all profile config templates (.finance, .design, .payments, .relations, .brain)
- Translate all profile cron JSON files to English
- Translate Strategist, Diplomat, and Brain Python tools to English with aligned keys
- Translate data/cron.json and data/tasks.json to English
- Update MISSING_IMPLEMENTATION.md with current gaps
- Verify demo script, dashboard build, and Python syntax
</commit_message>
<xml_diff>
--- a/data/sample_expenses.xlsx
+++ b/data/sample_expenses.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Income" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
refactor(i18n): remove legacy Spanish aliases from Diplomat CRM and include dashboard UI translations
</commit_message>
<xml_diff>
--- a/data/sample_expenses.xlsx
+++ b/data/sample_expenses.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Income" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
docs: final review polish — README badges, internal links, for-developers cross-references, and updated memory
</commit_message>
<xml_diff>
--- a/data/sample_expenses.xlsx
+++ b/data/sample_expenses.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Income" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
docs(hero-guide): normalize remaining python command to python3
</commit_message>
<xml_diff>
--- a/data/sample_expenses.xlsx
+++ b/data/sample_expenses.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Income" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
docs: final consistency pass — CHANGELOG update and regenerated demo artifacts
</commit_message>
<xml_diff>
--- a/data/sample_expenses.xlsx
+++ b/data/sample_expenses.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Income" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
fix: replace fastmcp with mcp in requirements, add python 3.10+ detection to install.sh
</commit_message>
<xml_diff>
--- a/data/sample_expenses.xlsx
+++ b/data/sample_expenses.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Income" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
cleanup: phase 0 contaminants cleanup
- Delete dead code/stubs: Kimi_Agent_10 Storytelling Web Sites, examples/*-stub.py,
  docs/PARTENON_GUIDE.html, docs/HERMES_GATEWAY_AUDIT.md, old superpowers plans/specs
- Anonymize sample data: onboarding engine, clients.json, HERO_GUIDE, workshop
  simulations, vendor/client templates (use *.example.test domains and generic names)
- Harden dashboard auth: remove admin/partenon fallbacks, require DASHBOARD_AUTH_SECRET
- Replace external gbrain binary dependency with local GBrainStore
- Add LICENSE, CONTRIBUTING.md, SECURITY.md, NOTICE.md
- Update TODOS.md and .gitignore for generated artifacts
</commit_message>
<xml_diff>
--- a/data/sample_expenses.xlsx
+++ b/data/sample_expenses.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Income" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
chore(phase-0): complete contaminants cleanup, secure installer, and CI
</commit_message>
<xml_diff>
--- a/data/sample_expenses.xlsx
+++ b/data/sample_expenses.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Income" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
docs(hermes): add operating modes, MCP tools, and dry-run/live tables to all hero profiles
</commit_message>
<xml_diff>
--- a/data/sample_expenses.xlsx
+++ b/data/sample_expenses.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Income" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat(phase-2): complete hero final design + MCP wrappers
- Finalize dry-run/live tool lists for all 7 heroes.
- Rewrite SOUL.md and SKILL.md per hero with operating modes, MCP catalogs, and dry-run/live tables.
- Implement dry-run wrappers in every MCP server (memory, finance, payments, comms, security, ops, relations).
- Add 6 collaboration handoff workflows to workflow_engine.py.
- Add tests/test_mcp_servers.py and tests/test_handoffs.py (27 tests passing).
- Update TODOS.md, CHANGELOG.md, MEMORY.md, PROGRESS.md, and brain central.
</commit_message>
<xml_diff>
--- a/data/sample_expenses.xlsx
+++ b/data/sample_expenses.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Income" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fixed Expenses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Variable Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Suppliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>